<commit_message>
Cập nhật biểu mẫu thống kê và bổ sung công cụ tra cứu mật khẩu
</commit_message>
<xml_diff>
--- a/KnowledgeSystem/AppResources/317/Templates/TE-701-T001-01 技術工程師評鑑學科成績明細表.xlsx
+++ b/KnowledgeSystem/AppResources/317/Templates/TE-701-T001-01 技術工程師評鑑學科成績明細表.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\1.經理室\00組務\00歷年文件\6.張氏水\2026年技術工程師評鑑 作業標準修訂\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\01. DEV\01.7System\01.Projects\7system\KnowledgeSystem\AppResources\317\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6C5BFA6-8CAA-42DB-894A-4974F847468C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20400" windowHeight="7245"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -19,15 +20,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>VNW0012995</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>技術工程師評鑑學科成績明細表</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -183,30 +184,6 @@
       <t>學科成績</t>
     </r>
     <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>經理室管理組</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="標楷體"/>
-        <family val="4"/>
-        <charset val="136"/>
-      </rPr>
-      <t>張氏水</t>
-    </r>
   </si>
   <si>
     <r>
@@ -285,8 +262,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="11">
     <font>
       <sz val="13"/>
       <color theme="1"/>
@@ -350,16 +327,13 @@
     </font>
     <font>
       <sz val="14"/>
-      <color rgb="FFFF0000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color rgb="FFFF0000"/>
-      <name val="標楷體"/>
-      <family val="4"/>
-      <charset val="136"/>
+      <sz val="13"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -436,27 +410,27 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -488,7 +462,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="圖片 2"/>
+        <xdr:cNvPr id="2" name="圖片 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -793,12 +773,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="18.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.88671875" style="1" bestFit="1" customWidth="1"/>
@@ -809,153 +789,150 @@
     <col min="7" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="17.25">
       <c r="E1" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="21" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="21">
+      <c r="A2" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="6"/>
+    </row>
+    <row r="3" spans="1:6" ht="21">
+      <c r="A3" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="6"/>
+    </row>
+    <row r="4" spans="1:6" ht="19.5">
+      <c r="A4" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="11"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="11"/>
+    </row>
+    <row r="5" spans="1:6" ht="39">
+      <c r="A5" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="6"/>
-    </row>
-    <row r="3" spans="1:6" ht="21" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="6"/>
-    </row>
-    <row r="4" spans="1:6" ht="19.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+      <c r="B5" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="1:6" ht="18.75">
+      <c r="A6" s="12"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7" spans="1:6" ht="18.75">
+      <c r="A7" s="12"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" spans="1:6" ht="18.75">
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="5"/>
+    </row>
+    <row r="9" spans="1:6" ht="18.75">
+      <c r="A9" s="13"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="5"/>
+    </row>
+    <row r="10" spans="1:6" ht="18.75">
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="5"/>
+    </row>
+    <row r="11" spans="1:6" ht="18.75">
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="5"/>
+    </row>
+    <row r="12" spans="1:6" ht="18.75">
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="5"/>
+    </row>
+    <row r="13" spans="1:6" ht="18.75">
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="5"/>
+    </row>
+    <row r="14" spans="1:6" ht="18.75">
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="5"/>
+    </row>
+    <row r="15" spans="1:6" ht="18.75">
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="5"/>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="14"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+    </row>
+    <row r="17" spans="5:5" ht="17.25">
+      <c r="E17" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="14"/>
-    </row>
-    <row r="5" spans="1:6" ht="39" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" s="3"/>
-    </row>
-    <row r="6" spans="1:6" ht="19.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="9">
-        <v>7010</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="9">
-        <v>89</v>
-      </c>
-      <c r="F6" s="4"/>
-    </row>
-    <row r="7" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="10"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="4"/>
-    </row>
-    <row r="8" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="11"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="5"/>
-    </row>
-    <row r="9" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="11"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="5"/>
-    </row>
-    <row r="10" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="11"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="5"/>
-    </row>
-    <row r="11" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="5"/>
-    </row>
-    <row r="12" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="5"/>
-    </row>
-    <row r="13" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="5"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="5"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="5"/>
-    </row>
-    <row r="17" spans="5:5" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="E17" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>